<commit_message>
fix: replace placeholder MK 0 enhancement data with real Bane/Havoc/Scourge tiers, map correct materials
</commit_message>
<xml_diff>
--- a/src/data/excel/Behemoth_Enhancements_FINAL.xlsx
+++ b/src/data/excel/Behemoth_Enhancements_FINAL.xlsx
@@ -5,10 +5,10 @@
   <sheets>
     <sheet name="MK III" sheetId="1" r:id="rId1"/>
     <sheet name="MK IV" sheetId="2" r:id="rId2"/>
-    <sheet name="MK 0" sheetId="3" r:id="rId3"/>
-    <sheet name="MK I" sheetId="4" r:id="rId4"/>
-    <sheet name="MK II" sheetId="5" r:id="rId5"/>
-    <sheet name="MK V" sheetId="6" r:id="rId6"/>
+    <sheet name="MK I" sheetId="3" r:id="rId3"/>
+    <sheet name="MK II" sheetId="4" r:id="rId4"/>
+    <sheet name="MK V" sheetId="5" r:id="rId5"/>
+    <sheet name="MK 0" sheetId="6" r:id="rId6"/>
   </sheets>
 </workbook>
 </file>
@@ -8437,7 +8437,19 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:J66"/>
+  <cols>
+    <col min="1" max="1" width="20.83203125" customWidth="1"/>
+    <col min="2" max="2" width="22.83203125" customWidth="1"/>
+    <col min="3" max="3" width="15.83203125" customWidth="1"/>
+    <col min="4" max="4" width="15.83203125" customWidth="1"/>
+    <col min="5" max="5" width="15.83203125" customWidth="1"/>
+    <col min="6" max="6" width="15.83203125" customWidth="1"/>
+    <col min="7" max="7" width="15.83203125" customWidth="1"/>
+    <col min="8" max="8" width="15.83203125" customWidth="1"/>
+    <col min="9" max="9" width="25.83203125" customWidth="1"/>
+    <col min="10" max="10" width="20.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -8472,168 +8484,2088 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2">
-        <v>1</v>
+      <c r="A2" t="str">
+        <v>Bane 1</v>
       </c>
       <c r="B2" t="str">
-        <v>Level 1</v>
+        <v>Infantry Lethality</v>
       </c>
       <c r="C2">
-        <v>0.01</v>
-      </c>
-      <c r="D2">
-        <v>0.01</v>
-      </c>
-      <c r="E2">
-        <v>0.01</v>
-      </c>
-      <c r="F2">
-        <v>0.01</v>
-      </c>
-      <c r="G2">
-        <v>0.01</v>
-      </c>
-      <c r="H2">
-        <v>0.01</v>
+        <v>0.006</v>
+      </c>
+      <c r="D2" t="str">
+        <v/>
+      </c>
+      <c r="E2" t="str">
+        <v/>
+      </c>
+      <c r="F2" t="str">
+        <v/>
+      </c>
+      <c r="G2" t="str">
+        <v/>
+      </c>
+      <c r="H2" t="str">
+        <v/>
       </c>
       <c r="I2" t="str">
-        <v/>
-      </c>
-      <c r="J2">
+        <v>Construction Time</v>
+      </c>
+      <c r="J2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Bane 2</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Infantry Health</v>
+      </c>
+      <c r="C3">
+        <v>0.006</v>
+      </c>
+      <c r="D3">
+        <v>0.006</v>
+      </c>
+      <c r="E3" t="str">
+        <v/>
+      </c>
+      <c r="F3" t="str">
+        <v/>
+      </c>
+      <c r="G3" t="str">
+        <v/>
+      </c>
+      <c r="H3" t="str">
+        <v/>
+      </c>
+      <c r="I3" t="str">
+        <v>Research Progress</v>
+      </c>
+      <c r="J3">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Bane 3</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Rider Lethality</v>
+      </c>
+      <c r="C4">
+        <v>0.006</v>
+      </c>
+      <c r="D4">
+        <v>0.006</v>
+      </c>
+      <c r="E4">
+        <v>0.006</v>
+      </c>
+      <c r="F4" t="str">
+        <v/>
+      </c>
+      <c r="G4" t="str">
+        <v/>
+      </c>
+      <c r="H4" t="str">
+        <v/>
+      </c>
+      <c r="I4" t="str">
+        <v>Speedy Training</v>
+      </c>
+      <c r="J4">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Bane 4</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Rider Health</v>
+      </c>
+      <c r="C5">
+        <v>0.006</v>
+      </c>
+      <c r="D5">
+        <v>0.006</v>
+      </c>
+      <c r="E5">
+        <v>0.006</v>
+      </c>
+      <c r="F5">
+        <v>0.006</v>
+      </c>
+      <c r="G5" t="str">
+        <v/>
+      </c>
+      <c r="H5" t="str">
+        <v/>
+      </c>
+      <c r="I5" t="str">
+        <v>Wood Gathering</v>
+      </c>
+      <c r="J5">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Bane 5</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Hunter Lethality</v>
+      </c>
+      <c r="C6">
+        <v>0.006</v>
+      </c>
+      <c r="D6">
+        <v>0.006</v>
+      </c>
+      <c r="E6">
+        <v>0.006</v>
+      </c>
+      <c r="F6">
+        <v>0.006</v>
+      </c>
+      <c r="G6">
+        <v>0.006</v>
+      </c>
+      <c r="H6" t="str">
+        <v/>
+      </c>
+      <c r="I6" t="str">
+        <v>Building Materials</v>
+      </c>
+      <c r="J6">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Bane 6</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Hunter Health</v>
+      </c>
+      <c r="C7">
+        <v>0.006</v>
+      </c>
+      <c r="D7">
+        <v>0.006</v>
+      </c>
+      <c r="E7">
+        <v>0.006</v>
+      </c>
+      <c r="F7">
+        <v>0.006</v>
+      </c>
+      <c r="G7">
+        <v>0.006</v>
+      </c>
+      <c r="H7">
+        <v>0.006</v>
+      </c>
+      <c r="I7" t="str">
+        <v/>
+      </c>
+      <c r="J7">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Bane 7</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Infantry Lethality</v>
+      </c>
+      <c r="C8">
+        <v>0.012</v>
+      </c>
+      <c r="D8">
+        <v>0.006</v>
+      </c>
+      <c r="E8">
+        <v>0.006</v>
+      </c>
+      <c r="F8">
+        <v>0.006</v>
+      </c>
+      <c r="G8">
+        <v>0.006</v>
+      </c>
+      <c r="H8">
+        <v>0.006</v>
+      </c>
+      <c r="I8" t="str">
+        <v>Training Resources</v>
+      </c>
+      <c r="J8">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Bane 8</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Infantry Health</v>
+      </c>
+      <c r="C9">
+        <v>0.012</v>
+      </c>
+      <c r="D9">
+        <v>0.012</v>
+      </c>
+      <c r="E9">
+        <v>0.006</v>
+      </c>
+      <c r="F9">
+        <v>0.006</v>
+      </c>
+      <c r="G9">
+        <v>0.006</v>
+      </c>
+      <c r="H9">
+        <v>0.006</v>
+      </c>
+      <c r="I9" t="str">
+        <v/>
+      </c>
+      <c r="J9">
         <v>15</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3">
-        <v>2</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Level 2</v>
-      </c>
-      <c r="C3">
-        <v>0.01</v>
-      </c>
-      <c r="D3">
-        <v>0.01</v>
-      </c>
-      <c r="E3">
-        <v>0.01</v>
-      </c>
-      <c r="F3">
-        <v>0.01</v>
-      </c>
-      <c r="G3">
-        <v>0.01</v>
-      </c>
-      <c r="H3">
-        <v>0.01</v>
-      </c>
-      <c r="I3" t="str">
-        <v/>
-      </c>
-      <c r="J3">
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Bane 9</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Rider Lethality</v>
+      </c>
+      <c r="C10">
+        <v>0.012</v>
+      </c>
+      <c r="D10">
+        <v>0.012</v>
+      </c>
+      <c r="E10">
+        <v>0.012</v>
+      </c>
+      <c r="F10">
+        <v>0.006</v>
+      </c>
+      <c r="G10">
+        <v>0.006</v>
+      </c>
+      <c r="H10">
+        <v>0.006</v>
+      </c>
+      <c r="I10" t="str">
+        <v>Metal Gathering</v>
+      </c>
+      <c r="J10">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>Bane 10</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Rider Health</v>
+      </c>
+      <c r="C11">
+        <v>0.012</v>
+      </c>
+      <c r="D11">
+        <v>0.012</v>
+      </c>
+      <c r="E11">
+        <v>0.012</v>
+      </c>
+      <c r="F11">
+        <v>0.012</v>
+      </c>
+      <c r="G11">
+        <v>0.006</v>
+      </c>
+      <c r="H11">
+        <v>0.006</v>
+      </c>
+      <c r="I11" t="str">
+        <v>Gas Gathering</v>
+      </c>
+      <c r="J11">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>Bane Ultra-Enhance</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Hunter Lethality</v>
+      </c>
+      <c r="C12">
+        <v>0.012</v>
+      </c>
+      <c r="D12">
+        <v>0.012</v>
+      </c>
+      <c r="E12">
+        <v>0.012</v>
+      </c>
+      <c r="F12">
+        <v>0.012</v>
+      </c>
+      <c r="G12">
+        <v>0.012</v>
+      </c>
+      <c r="H12">
+        <v>0.006</v>
+      </c>
+      <c r="I12" t="str">
+        <v/>
+      </c>
+      <c r="J12">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>Havoc I 1</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Hunter Lethality</v>
+      </c>
+      <c r="C13" t="str">
+        <v/>
+      </c>
+      <c r="D13" t="str">
+        <v/>
+      </c>
+      <c r="E13" t="str">
+        <v/>
+      </c>
+      <c r="F13" t="str">
+        <v/>
+      </c>
+      <c r="G13">
+        <v>0.012</v>
+      </c>
+      <c r="H13" t="str">
+        <v/>
+      </c>
+      <c r="I13" t="str">
+        <v>Infantry Attack</v>
+      </c>
+      <c r="J13" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>Havoc I 2</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Hunter Health</v>
+      </c>
+      <c r="C14" t="str">
+        <v/>
+      </c>
+      <c r="D14" t="str">
+        <v/>
+      </c>
+      <c r="E14" t="str">
+        <v/>
+      </c>
+      <c r="F14" t="str">
+        <v/>
+      </c>
+      <c r="G14">
+        <v>0.012</v>
+      </c>
+      <c r="H14">
+        <v>0.012</v>
+      </c>
+      <c r="I14" t="str">
+        <v>Rider Defense</v>
+      </c>
+      <c r="J14">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>Havoc I 3</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Infantry Lethality</v>
+      </c>
+      <c r="C15">
+        <v>0.018000000000000002</v>
+      </c>
+      <c r="D15" t="str">
+        <v/>
+      </c>
+      <c r="E15" t="str">
+        <v/>
+      </c>
+      <c r="F15" t="str">
+        <v/>
+      </c>
+      <c r="G15">
+        <v>0.012</v>
+      </c>
+      <c r="H15">
+        <v>0.012</v>
+      </c>
+      <c r="I15" t="str">
+        <v>Hunter Defense</v>
+      </c>
+      <c r="J15">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>Havoc I 4</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Infantry Health</v>
+      </c>
+      <c r="C16">
+        <v>0.018000000000000002</v>
+      </c>
+      <c r="D16">
+        <v>0.018000000000000002</v>
+      </c>
+      <c r="E16" t="str">
+        <v/>
+      </c>
+      <c r="F16" t="str">
+        <v/>
+      </c>
+      <c r="G16">
+        <v>0.012</v>
+      </c>
+      <c r="H16">
+        <v>0.012</v>
+      </c>
+      <c r="I16" t="str">
+        <v>Infantry Defense</v>
+      </c>
+      <c r="J16">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>Havoc I 5</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Rider Lethality</v>
+      </c>
+      <c r="C17">
+        <v>0.018000000000000002</v>
+      </c>
+      <c r="D17">
+        <v>0.018000000000000002</v>
+      </c>
+      <c r="E17">
+        <v>0.018000000000000002</v>
+      </c>
+      <c r="F17" t="str">
+        <v/>
+      </c>
+      <c r="G17">
+        <v>0.012</v>
+      </c>
+      <c r="H17">
+        <v>0.012</v>
+      </c>
+      <c r="I17" t="str">
+        <v/>
+      </c>
+      <c r="J17">
         <v>20</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4">
-        <v>3</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Level 3</v>
-      </c>
-      <c r="C4">
-        <v>0.01</v>
-      </c>
-      <c r="D4">
-        <v>0.01</v>
-      </c>
-      <c r="E4">
-        <v>0.01</v>
-      </c>
-      <c r="F4">
-        <v>0.01</v>
-      </c>
-      <c r="G4">
-        <v>0.01</v>
-      </c>
-      <c r="H4">
-        <v>0.01</v>
-      </c>
-      <c r="I4" t="str">
-        <v/>
-      </c>
-      <c r="J4">
+    <row r="18">
+      <c r="A18" t="str">
+        <v>Havoc I 6</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Rider Health</v>
+      </c>
+      <c r="C18">
+        <v>0.018000000000000002</v>
+      </c>
+      <c r="D18">
+        <v>0.018000000000000002</v>
+      </c>
+      <c r="E18">
+        <v>0.018000000000000002</v>
+      </c>
+      <c r="F18">
+        <v>0.018000000000000002</v>
+      </c>
+      <c r="G18">
+        <v>0.012</v>
+      </c>
+      <c r="H18">
+        <v>0.012</v>
+      </c>
+      <c r="I18" t="str">
+        <v>Rider Attack</v>
+      </c>
+      <c r="J18">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>Havoc I 7</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Hunter Lethality</v>
+      </c>
+      <c r="C19">
+        <v>0.018000000000000002</v>
+      </c>
+      <c r="D19">
+        <v>0.018000000000000002</v>
+      </c>
+      <c r="E19">
+        <v>0.018000000000000002</v>
+      </c>
+      <c r="F19">
+        <v>0.018000000000000002</v>
+      </c>
+      <c r="G19">
+        <v>0.018000000000000002</v>
+      </c>
+      <c r="H19">
+        <v>0.012</v>
+      </c>
+      <c r="I19" t="str">
+        <v/>
+      </c>
+      <c r="J19">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>Havoc I 8</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Hunter Health</v>
+      </c>
+      <c r="C20">
+        <v>0.018000000000000002</v>
+      </c>
+      <c r="D20">
+        <v>0.018000000000000002</v>
+      </c>
+      <c r="E20">
+        <v>0.018000000000000002</v>
+      </c>
+      <c r="F20">
+        <v>0.018000000000000002</v>
+      </c>
+      <c r="G20">
+        <v>0.018000000000000002</v>
+      </c>
+      <c r="H20">
+        <v>0.018000000000000002</v>
+      </c>
+      <c r="I20" t="str">
+        <v>Hunter Attack</v>
+      </c>
+      <c r="J20">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>Havoc I 9</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Infantry Lethality</v>
+      </c>
+      <c r="C21">
+        <v>0.024</v>
+      </c>
+      <c r="D21">
+        <v>0.018000000000000002</v>
+      </c>
+      <c r="E21">
+        <v>0.018000000000000002</v>
+      </c>
+      <c r="F21">
+        <v>0.018000000000000002</v>
+      </c>
+      <c r="G21">
+        <v>0.018000000000000002</v>
+      </c>
+      <c r="H21">
+        <v>0.018000000000000002</v>
+      </c>
+      <c r="I21" t="str">
+        <v/>
+      </c>
+      <c r="J21">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>Havoc I 10</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Infantry Health</v>
+      </c>
+      <c r="C22">
+        <v>0.024</v>
+      </c>
+      <c r="D22">
+        <v>0.024</v>
+      </c>
+      <c r="E22">
+        <v>0.018000000000000002</v>
+      </c>
+      <c r="F22">
+        <v>0.018000000000000002</v>
+      </c>
+      <c r="G22">
+        <v>0.018000000000000002</v>
+      </c>
+      <c r="H22">
+        <v>0.018000000000000002</v>
+      </c>
+      <c r="I22" t="str">
+        <v>Infantry Lethality</v>
+      </c>
+      <c r="J22">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>Havoc I Ultra-Enhance</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Rider Lethality</v>
+      </c>
+      <c r="C23">
+        <v>0.024</v>
+      </c>
+      <c r="D23">
+        <v>0.024</v>
+      </c>
+      <c r="E23">
+        <v>0.024</v>
+      </c>
+      <c r="F23">
+        <v>0.018000000000000002</v>
+      </c>
+      <c r="G23">
+        <v>0.018000000000000002</v>
+      </c>
+      <c r="H23">
+        <v>0.018000000000000002</v>
+      </c>
+      <c r="I23" t="str">
+        <v/>
+      </c>
+      <c r="J23">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>Havoc II 1</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Rider Lethality</v>
+      </c>
+      <c r="C24" t="str">
+        <v/>
+      </c>
+      <c r="D24" t="str">
+        <v/>
+      </c>
+      <c r="E24">
+        <v>0.024</v>
+      </c>
+      <c r="F24" t="str">
+        <v/>
+      </c>
+      <c r="G24" t="str">
+        <v/>
+      </c>
+      <c r="H24" t="str">
+        <v/>
+      </c>
+      <c r="I24" t="str">
+        <v/>
+      </c>
+      <c r="J24" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>Havoc II 2</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Rider Health</v>
+      </c>
+      <c r="C25" t="str">
+        <v/>
+      </c>
+      <c r="D25" t="str">
+        <v/>
+      </c>
+      <c r="E25">
+        <v>0.024</v>
+      </c>
+      <c r="F25">
+        <v>0.024</v>
+      </c>
+      <c r="G25" t="str">
+        <v/>
+      </c>
+      <c r="H25" t="str">
+        <v/>
+      </c>
+      <c r="I25" t="str">
+        <v>Rider Health</v>
+      </c>
+      <c r="J25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>Havoc II 3</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Hunter Lethality</v>
+      </c>
+      <c r="C26" t="str">
+        <v/>
+      </c>
+      <c r="D26" t="str">
+        <v/>
+      </c>
+      <c r="E26">
+        <v>0.024</v>
+      </c>
+      <c r="F26">
+        <v>0.024</v>
+      </c>
+      <c r="G26">
+        <v>0.024</v>
+      </c>
+      <c r="H26" t="str">
+        <v/>
+      </c>
+      <c r="I26" t="str">
+        <v/>
+      </c>
+      <c r="J26">
         <v>25</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5">
-        <v>4</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Level 4</v>
-      </c>
-      <c r="C5">
-        <v>0.01</v>
-      </c>
-      <c r="D5">
-        <v>0.01</v>
-      </c>
-      <c r="E5">
-        <v>0.01</v>
-      </c>
-      <c r="F5">
-        <v>0.01</v>
-      </c>
-      <c r="G5">
-        <v>0.01</v>
-      </c>
-      <c r="H5">
-        <v>0.01</v>
-      </c>
-      <c r="I5" t="str">
-        <v/>
-      </c>
-      <c r="J5">
+    <row r="27">
+      <c r="A27" t="str">
+        <v>Havoc II 4</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Hunter Health</v>
+      </c>
+      <c r="C27" t="str">
+        <v/>
+      </c>
+      <c r="D27" t="str">
+        <v/>
+      </c>
+      <c r="E27">
+        <v>0.024</v>
+      </c>
+      <c r="F27">
+        <v>0.024</v>
+      </c>
+      <c r="G27">
+        <v>0.024</v>
+      </c>
+      <c r="H27">
+        <v>0.024</v>
+      </c>
+      <c r="I27" t="str">
+        <v>Hunter Health</v>
+      </c>
+      <c r="J27">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>Havoc II 5</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Infantry Lethality</v>
+      </c>
+      <c r="C28">
+        <v>0.03</v>
+      </c>
+      <c r="D28" t="str">
+        <v/>
+      </c>
+      <c r="E28">
+        <v>0.024</v>
+      </c>
+      <c r="F28">
+        <v>0.024</v>
+      </c>
+      <c r="G28">
+        <v>0.024</v>
+      </c>
+      <c r="H28">
+        <v>0.024</v>
+      </c>
+      <c r="I28" t="str">
+        <v/>
+      </c>
+      <c r="J28">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>Havoc II 6</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Infantry Health</v>
+      </c>
+      <c r="C29">
+        <v>0.03</v>
+      </c>
+      <c r="D29">
+        <v>0.03</v>
+      </c>
+      <c r="E29">
+        <v>0.024</v>
+      </c>
+      <c r="F29">
+        <v>0.024</v>
+      </c>
+      <c r="G29">
+        <v>0.024</v>
+      </c>
+      <c r="H29">
+        <v>0.024</v>
+      </c>
+      <c r="I29" t="str">
+        <v>Infantry Health</v>
+      </c>
+      <c r="J29">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>Havoc II 7</v>
+      </c>
+      <c r="B30" t="str">
+        <v>Rider Lethality</v>
+      </c>
+      <c r="C30">
+        <v>0.03</v>
+      </c>
+      <c r="D30">
+        <v>0.03</v>
+      </c>
+      <c r="E30">
+        <v>0.03</v>
+      </c>
+      <c r="F30">
+        <v>0.024</v>
+      </c>
+      <c r="G30">
+        <v>0.024</v>
+      </c>
+      <c r="H30">
+        <v>0.024</v>
+      </c>
+      <c r="I30" t="str">
+        <v/>
+      </c>
+      <c r="J30">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>Havoc II 8</v>
+      </c>
+      <c r="B31" t="str">
+        <v>Rider Health</v>
+      </c>
+      <c r="C31">
+        <v>0.03</v>
+      </c>
+      <c r="D31">
+        <v>0.03</v>
+      </c>
+      <c r="E31">
+        <v>0.03</v>
+      </c>
+      <c r="F31">
+        <v>0.03</v>
+      </c>
+      <c r="G31">
+        <v>0.024</v>
+      </c>
+      <c r="H31">
+        <v>0.024</v>
+      </c>
+      <c r="I31" t="str">
+        <v>Rider Lethality</v>
+      </c>
+      <c r="J31">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>Havoc II 9</v>
+      </c>
+      <c r="B32" t="str">
+        <v>Hunter Lethality</v>
+      </c>
+      <c r="C32">
+        <v>0.03</v>
+      </c>
+      <c r="D32">
+        <v>0.03</v>
+      </c>
+      <c r="E32">
+        <v>0.03</v>
+      </c>
+      <c r="F32">
+        <v>0.03</v>
+      </c>
+      <c r="G32">
+        <v>0.03</v>
+      </c>
+      <c r="H32">
+        <v>0.024</v>
+      </c>
+      <c r="I32" t="str">
+        <v/>
+      </c>
+      <c r="J32">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>Havoc II 10</v>
+      </c>
+      <c r="B33" t="str">
+        <v>Hunter Health</v>
+      </c>
+      <c r="C33">
+        <v>0.03</v>
+      </c>
+      <c r="D33">
+        <v>0.03</v>
+      </c>
+      <c r="E33">
+        <v>0.03</v>
+      </c>
+      <c r="F33">
+        <v>0.03</v>
+      </c>
+      <c r="G33">
+        <v>0.03</v>
+      </c>
+      <c r="H33">
+        <v>0.03</v>
+      </c>
+      <c r="I33" t="str">
+        <v>Hunter Lethality</v>
+      </c>
+      <c r="J33">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>Havoc II Ultra-Enhance</v>
+      </c>
+      <c r="B34" t="str">
+        <v>Infantry Lethality</v>
+      </c>
+      <c r="C34">
+        <v>0.036000000000000004</v>
+      </c>
+      <c r="D34">
+        <v>0.03</v>
+      </c>
+      <c r="E34">
+        <v>0.03</v>
+      </c>
+      <c r="F34">
+        <v>0.03</v>
+      </c>
+      <c r="G34">
+        <v>0.03</v>
+      </c>
+      <c r="H34">
+        <v>0.03</v>
+      </c>
+      <c r="I34" t="str">
+        <v/>
+      </c>
+      <c r="J34">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>Scourge I 1</v>
+      </c>
+      <c r="B35" t="str">
+        <v>Infantry Lethality</v>
+      </c>
+      <c r="C35">
+        <v>0.036000000000000004</v>
+      </c>
+      <c r="D35" t="str">
+        <v/>
+      </c>
+      <c r="E35" t="str">
+        <v/>
+      </c>
+      <c r="F35" t="str">
+        <v/>
+      </c>
+      <c r="G35" t="str">
+        <v/>
+      </c>
+      <c r="H35" t="str">
+        <v/>
+      </c>
+      <c r="I35" t="str">
+        <v>Active Strike</v>
+      </c>
+      <c r="J35" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>Scourge I 2</v>
+      </c>
+      <c r="B36" t="str">
+        <v>Infantry Health</v>
+      </c>
+      <c r="C36">
+        <v>0.036000000000000004</v>
+      </c>
+      <c r="D36">
+        <v>0.036000000000000004</v>
+      </c>
+      <c r="E36" t="str">
+        <v/>
+      </c>
+      <c r="F36" t="str">
+        <v/>
+      </c>
+      <c r="G36" t="str">
+        <v/>
+      </c>
+      <c r="H36" t="str">
+        <v/>
+      </c>
+      <c r="I36" t="str">
+        <v/>
+      </c>
+      <c r="J36">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>Scourge I 3</v>
+      </c>
+      <c r="B37" t="str">
+        <v>Rider Lethality</v>
+      </c>
+      <c r="C37">
+        <v>0.036000000000000004</v>
+      </c>
+      <c r="D37">
+        <v>0.036000000000000004</v>
+      </c>
+      <c r="E37">
+        <v>0.036000000000000004</v>
+      </c>
+      <c r="F37" t="str">
+        <v/>
+      </c>
+      <c r="G37" t="str">
+        <v/>
+      </c>
+      <c r="H37" t="str">
+        <v/>
+      </c>
+      <c r="I37" t="str">
+        <v/>
+      </c>
+      <c r="J37">
         <v>30</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6">
-        <v>5</v>
-      </c>
-      <c r="B6" t="str">
-        <v>Level 5</v>
-      </c>
-      <c r="C6">
-        <v>0.01</v>
-      </c>
-      <c r="D6">
-        <v>0.01</v>
-      </c>
-      <c r="E6">
-        <v>0.01</v>
-      </c>
-      <c r="F6">
-        <v>0.01</v>
-      </c>
-      <c r="G6">
-        <v>0.01</v>
-      </c>
-      <c r="H6">
-        <v>0.01</v>
-      </c>
-      <c r="I6" t="str">
-        <v/>
-      </c>
-      <c r="J6">
+    <row r="38">
+      <c r="A38" t="str">
+        <v>Scourge I 4</v>
+      </c>
+      <c r="B38" t="str">
+        <v>Rider Health</v>
+      </c>
+      <c r="C38">
+        <v>0.036000000000000004</v>
+      </c>
+      <c r="D38">
+        <v>0.036000000000000004</v>
+      </c>
+      <c r="E38">
+        <v>0.036000000000000004</v>
+      </c>
+      <c r="F38">
+        <v>0.036000000000000004</v>
+      </c>
+      <c r="G38" t="str">
+        <v/>
+      </c>
+      <c r="H38" t="str">
+        <v/>
+      </c>
+      <c r="I38" t="str">
+        <v>Troop Attack</v>
+      </c>
+      <c r="J38">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>Scourge I 5</v>
+      </c>
+      <c r="B39" t="str">
+        <v>Hunter Lethality</v>
+      </c>
+      <c r="C39">
+        <v>0.036000000000000004</v>
+      </c>
+      <c r="D39">
+        <v>0.036000000000000004</v>
+      </c>
+      <c r="E39">
+        <v>0.036000000000000004</v>
+      </c>
+      <c r="F39">
+        <v>0.036000000000000004</v>
+      </c>
+      <c r="G39">
+        <v>0.036000000000000004</v>
+      </c>
+      <c r="H39" t="str">
+        <v/>
+      </c>
+      <c r="I39" t="str">
+        <v/>
+      </c>
+      <c r="J39">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>Scourge I 6</v>
+      </c>
+      <c r="B40" t="str">
+        <v>Hunter Health</v>
+      </c>
+      <c r="C40">
+        <v>0.036000000000000004</v>
+      </c>
+      <c r="D40">
+        <v>0.036000000000000004</v>
+      </c>
+      <c r="E40">
+        <v>0.036000000000000004</v>
+      </c>
+      <c r="F40">
+        <v>0.036000000000000004</v>
+      </c>
+      <c r="G40">
+        <v>0.036000000000000004</v>
+      </c>
+      <c r="H40">
+        <v>0.036000000000000004</v>
+      </c>
+      <c r="I40" t="str">
+        <v/>
+      </c>
+      <c r="J40">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>Scourge I 7</v>
+      </c>
+      <c r="B41" t="str">
+        <v>Infantry Lethality</v>
+      </c>
+      <c r="C41">
+        <v>0.042</v>
+      </c>
+      <c r="D41">
+        <v>0.036000000000000004</v>
+      </c>
+      <c r="E41">
+        <v>0.036000000000000004</v>
+      </c>
+      <c r="F41">
+        <v>0.036000000000000004</v>
+      </c>
+      <c r="G41">
+        <v>0.036000000000000004</v>
+      </c>
+      <c r="H41">
+        <v>0.036000000000000004</v>
+      </c>
+      <c r="I41" t="str">
+        <v>Rally Attack</v>
+      </c>
+      <c r="J41">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>Scourge I 8</v>
+      </c>
+      <c r="B42" t="str">
+        <v>Infantry Health</v>
+      </c>
+      <c r="C42">
+        <v>0.042</v>
+      </c>
+      <c r="D42">
+        <v>0.042</v>
+      </c>
+      <c r="E42">
+        <v>0.036000000000000004</v>
+      </c>
+      <c r="F42">
+        <v>0.036000000000000004</v>
+      </c>
+      <c r="G42">
+        <v>0.036000000000000004</v>
+      </c>
+      <c r="H42">
+        <v>0.036000000000000004</v>
+      </c>
+      <c r="I42" t="str">
+        <v/>
+      </c>
+      <c r="J42">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>Scourge I 9</v>
+      </c>
+      <c r="B43" t="str">
+        <v>Rider Lethality</v>
+      </c>
+      <c r="C43">
+        <v>0.042</v>
+      </c>
+      <c r="D43">
+        <v>0.042</v>
+      </c>
+      <c r="E43">
+        <v>0.042</v>
+      </c>
+      <c r="F43">
+        <v>0.036000000000000004</v>
+      </c>
+      <c r="G43">
+        <v>0.036000000000000004</v>
+      </c>
+      <c r="H43">
+        <v>0.036000000000000004</v>
+      </c>
+      <c r="I43" t="str">
+        <v/>
+      </c>
+      <c r="J43">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>Scourge I 10</v>
+      </c>
+      <c r="B44" t="str">
+        <v>Rider Health</v>
+      </c>
+      <c r="C44">
+        <v>0.042</v>
+      </c>
+      <c r="D44">
+        <v>0.042</v>
+      </c>
+      <c r="E44">
+        <v>0.042</v>
+      </c>
+      <c r="F44">
+        <v>0.042</v>
+      </c>
+      <c r="G44">
+        <v>0.036000000000000004</v>
+      </c>
+      <c r="H44">
+        <v>0.036000000000000004</v>
+      </c>
+      <c r="I44" t="str">
+        <v>Troop Lethality</v>
+      </c>
+      <c r="J44">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>Scourge I Ultra-Enhance</v>
+      </c>
+      <c r="B45" t="str">
+        <v>Hunter Lethality</v>
+      </c>
+      <c r="C45">
+        <v>0.042</v>
+      </c>
+      <c r="D45">
+        <v>0.042</v>
+      </c>
+      <c r="E45">
+        <v>0.042</v>
+      </c>
+      <c r="F45">
+        <v>0.042</v>
+      </c>
+      <c r="G45">
+        <v>0.042</v>
+      </c>
+      <c r="H45">
+        <v>0.036000000000000004</v>
+      </c>
+      <c r="I45" t="str">
+        <v/>
+      </c>
+      <c r="J45">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>Scourge II 1</v>
+      </c>
+      <c r="B46" t="str">
+        <v>Hunter Lethality</v>
+      </c>
+      <c r="C46" t="str">
+        <v/>
+      </c>
+      <c r="D46" t="str">
+        <v/>
+      </c>
+      <c r="E46" t="str">
+        <v/>
+      </c>
+      <c r="F46" t="str">
+        <v/>
+      </c>
+      <c r="G46">
+        <v>0.042</v>
+      </c>
+      <c r="H46" t="str">
+        <v/>
+      </c>
+      <c r="I46" t="str">
+        <v/>
+      </c>
+      <c r="J46" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>Scourge II 2</v>
+      </c>
+      <c r="B47" t="str">
+        <v>Hunter Health</v>
+      </c>
+      <c r="C47" t="str">
+        <v/>
+      </c>
+      <c r="D47" t="str">
+        <v/>
+      </c>
+      <c r="E47" t="str">
+        <v/>
+      </c>
+      <c r="F47" t="str">
+        <v/>
+      </c>
+      <c r="G47">
+        <v>0.042</v>
+      </c>
+      <c r="H47">
+        <v>0.042</v>
+      </c>
+      <c r="I47" t="str">
+        <v/>
+      </c>
+      <c r="J47">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>Scourge II 3</v>
+      </c>
+      <c r="B48" t="str">
+        <v>Infantry Lethality</v>
+      </c>
+      <c r="C48">
+        <v>0.048</v>
+      </c>
+      <c r="D48" t="str">
+        <v/>
+      </c>
+      <c r="E48" t="str">
+        <v/>
+      </c>
+      <c r="F48" t="str">
+        <v/>
+      </c>
+      <c r="G48">
+        <v>0.042</v>
+      </c>
+      <c r="H48">
+        <v>0.042</v>
+      </c>
+      <c r="I48" t="str">
+        <v>Rally Lethality</v>
+      </c>
+      <c r="J48">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>Scourge II 4</v>
+      </c>
+      <c r="B49" t="str">
+        <v>Infantry Health</v>
+      </c>
+      <c r="C49">
+        <v>0.048</v>
+      </c>
+      <c r="D49">
+        <v>0.048</v>
+      </c>
+      <c r="E49" t="str">
+        <v/>
+      </c>
+      <c r="F49" t="str">
+        <v/>
+      </c>
+      <c r="G49">
+        <v>0.042</v>
+      </c>
+      <c r="H49">
+        <v>0.042</v>
+      </c>
+      <c r="I49" t="str">
+        <v/>
+      </c>
+      <c r="J49">
         <v>35</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>Scourge II 5</v>
+      </c>
+      <c r="B50" t="str">
+        <v>Rider Lethality</v>
+      </c>
+      <c r="C50">
+        <v>0.048</v>
+      </c>
+      <c r="D50">
+        <v>0.048</v>
+      </c>
+      <c r="E50">
+        <v>0.048</v>
+      </c>
+      <c r="F50" t="str">
+        <v/>
+      </c>
+      <c r="G50">
+        <v>0.042</v>
+      </c>
+      <c r="H50">
+        <v>0.042</v>
+      </c>
+      <c r="I50" t="str">
+        <v/>
+      </c>
+      <c r="J50">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>Scourge II 6</v>
+      </c>
+      <c r="B51" t="str">
+        <v>Rider Health</v>
+      </c>
+      <c r="C51">
+        <v>0.048</v>
+      </c>
+      <c r="D51">
+        <v>0.048</v>
+      </c>
+      <c r="E51">
+        <v>0.048</v>
+      </c>
+      <c r="F51">
+        <v>0.048</v>
+      </c>
+      <c r="G51">
+        <v>0.042</v>
+      </c>
+      <c r="H51">
+        <v>0.042</v>
+      </c>
+      <c r="I51" t="str">
+        <v>Troop Defense</v>
+      </c>
+      <c r="J51">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>Scourge II 7</v>
+      </c>
+      <c r="B52" t="str">
+        <v>Hunter Lethality</v>
+      </c>
+      <c r="C52">
+        <v>0.048</v>
+      </c>
+      <c r="D52">
+        <v>0.048</v>
+      </c>
+      <c r="E52">
+        <v>0.048</v>
+      </c>
+      <c r="F52">
+        <v>0.048</v>
+      </c>
+      <c r="G52">
+        <v>0.048</v>
+      </c>
+      <c r="H52">
+        <v>0.042</v>
+      </c>
+      <c r="I52" t="str">
+        <v/>
+      </c>
+      <c r="J52">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>Scourge II 8</v>
+      </c>
+      <c r="B53" t="str">
+        <v>Hunter Health</v>
+      </c>
+      <c r="C53">
+        <v>0.048</v>
+      </c>
+      <c r="D53">
+        <v>0.048</v>
+      </c>
+      <c r="E53">
+        <v>0.048</v>
+      </c>
+      <c r="F53">
+        <v>0.048</v>
+      </c>
+      <c r="G53">
+        <v>0.048</v>
+      </c>
+      <c r="H53">
+        <v>0.048</v>
+      </c>
+      <c r="I53" t="str">
+        <v/>
+      </c>
+      <c r="J53">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>Scourge II 9</v>
+      </c>
+      <c r="B54" t="str">
+        <v>Infantry Lethality</v>
+      </c>
+      <c r="C54">
+        <v>0.054000000000000006</v>
+      </c>
+      <c r="D54">
+        <v>0.048</v>
+      </c>
+      <c r="E54">
+        <v>0.048</v>
+      </c>
+      <c r="F54">
+        <v>0.048</v>
+      </c>
+      <c r="G54">
+        <v>0.048</v>
+      </c>
+      <c r="H54">
+        <v>0.048</v>
+      </c>
+      <c r="I54" t="str">
+        <v>Rally Defense</v>
+      </c>
+      <c r="J54">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>Scourge II 10</v>
+      </c>
+      <c r="B55" t="str">
+        <v>Infantry Health</v>
+      </c>
+      <c r="C55">
+        <v>0.054000000000000006</v>
+      </c>
+      <c r="D55">
+        <v>0.054000000000000006</v>
+      </c>
+      <c r="E55">
+        <v>0.048</v>
+      </c>
+      <c r="F55">
+        <v>0.048</v>
+      </c>
+      <c r="G55">
+        <v>0.048</v>
+      </c>
+      <c r="H55">
+        <v>0.048</v>
+      </c>
+      <c r="I55" t="str">
+        <v/>
+      </c>
+      <c r="J55">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>Scourge II Ultra-Enhance</v>
+      </c>
+      <c r="B56" t="str">
+        <v>Rider Lethality</v>
+      </c>
+      <c r="C56">
+        <v>0.054000000000000006</v>
+      </c>
+      <c r="D56">
+        <v>0.054000000000000006</v>
+      </c>
+      <c r="E56">
+        <v>0.054000000000000006</v>
+      </c>
+      <c r="F56">
+        <v>0.048</v>
+      </c>
+      <c r="G56">
+        <v>0.048</v>
+      </c>
+      <c r="H56">
+        <v>0.048</v>
+      </c>
+      <c r="I56" t="str">
+        <v/>
+      </c>
+      <c r="J56">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>Scourge III 1</v>
+      </c>
+      <c r="B57" t="str">
+        <v>Rider Lethality</v>
+      </c>
+      <c r="C57" t="str">
+        <v/>
+      </c>
+      <c r="D57" t="str">
+        <v/>
+      </c>
+      <c r="E57">
+        <v>0.054000000000000006</v>
+      </c>
+      <c r="F57" t="str">
+        <v/>
+      </c>
+      <c r="G57" t="str">
+        <v/>
+      </c>
+      <c r="H57" t="str">
+        <v/>
+      </c>
+      <c r="I57" t="str">
+        <v/>
+      </c>
+      <c r="J57" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <v>Scourge III 2</v>
+      </c>
+      <c r="B58" t="str">
+        <v>Rider Health</v>
+      </c>
+      <c r="C58" t="str">
+        <v/>
+      </c>
+      <c r="D58" t="str">
+        <v/>
+      </c>
+      <c r="E58">
+        <v>0.054000000000000006</v>
+      </c>
+      <c r="F58">
+        <v>0.054000000000000006</v>
+      </c>
+      <c r="G58" t="str">
+        <v/>
+      </c>
+      <c r="H58" t="str">
+        <v/>
+      </c>
+      <c r="I58" t="str">
+        <v>Troop Health</v>
+      </c>
+      <c r="J58">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="str">
+        <v>Scourge III 3</v>
+      </c>
+      <c r="B59" t="str">
+        <v>Hunter Lethality</v>
+      </c>
+      <c r="C59" t="str">
+        <v/>
+      </c>
+      <c r="D59" t="str">
+        <v/>
+      </c>
+      <c r="E59">
+        <v>0.054000000000000006</v>
+      </c>
+      <c r="F59">
+        <v>0.054000000000000006</v>
+      </c>
+      <c r="G59">
+        <v>0.054000000000000006</v>
+      </c>
+      <c r="H59" t="str">
+        <v/>
+      </c>
+      <c r="I59" t="str">
+        <v/>
+      </c>
+      <c r="J59">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="str">
+        <v>Scourge III 4</v>
+      </c>
+      <c r="B60" t="str">
+        <v>Hunter Health</v>
+      </c>
+      <c r="C60" t="str">
+        <v/>
+      </c>
+      <c r="D60" t="str">
+        <v/>
+      </c>
+      <c r="E60">
+        <v>0.054000000000000006</v>
+      </c>
+      <c r="F60">
+        <v>0.054000000000000006</v>
+      </c>
+      <c r="G60">
+        <v>0.054000000000000006</v>
+      </c>
+      <c r="H60">
+        <v>0.054000000000000006</v>
+      </c>
+      <c r="I60" t="str">
+        <v/>
+      </c>
+      <c r="J60">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="str">
+        <v>Scourge III 5</v>
+      </c>
+      <c r="B61" t="str">
+        <v>Infantry Lethality</v>
+      </c>
+      <c r="C61">
+        <v>0.06</v>
+      </c>
+      <c r="D61" t="str">
+        <v/>
+      </c>
+      <c r="E61">
+        <v>0.054000000000000006</v>
+      </c>
+      <c r="F61">
+        <v>0.054000000000000006</v>
+      </c>
+      <c r="G61">
+        <v>0.054000000000000006</v>
+      </c>
+      <c r="H61">
+        <v>0.054000000000000006</v>
+      </c>
+      <c r="I61" t="str">
+        <v>Rally Health</v>
+      </c>
+      <c r="J61">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="str">
+        <v>Scourge III 6</v>
+      </c>
+      <c r="B62" t="str">
+        <v>Infantry Health</v>
+      </c>
+      <c r="C62">
+        <v>0.06</v>
+      </c>
+      <c r="D62">
+        <v>0.06</v>
+      </c>
+      <c r="E62">
+        <v>0.054000000000000006</v>
+      </c>
+      <c r="F62">
+        <v>0.054000000000000006</v>
+      </c>
+      <c r="G62">
+        <v>0.054000000000000006</v>
+      </c>
+      <c r="H62">
+        <v>0.054000000000000006</v>
+      </c>
+      <c r="I62" t="str">
+        <v/>
+      </c>
+      <c r="J62">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="str">
+        <v>Scourge III 7</v>
+      </c>
+      <c r="B63" t="str">
+        <v>Rider Lethality</v>
+      </c>
+      <c r="C63">
+        <v>0.06</v>
+      </c>
+      <c r="D63">
+        <v>0.06</v>
+      </c>
+      <c r="E63">
+        <v>0.06</v>
+      </c>
+      <c r="F63">
+        <v>0.054000000000000006</v>
+      </c>
+      <c r="G63">
+        <v>0.054000000000000006</v>
+      </c>
+      <c r="H63">
+        <v>0.054000000000000006</v>
+      </c>
+      <c r="I63" t="str">
+        <v>March Capacity</v>
+      </c>
+      <c r="J63">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="str">
+        <v>Scourge III 8</v>
+      </c>
+      <c r="B64" t="str">
+        <v>Rider Health</v>
+      </c>
+      <c r="C64">
+        <v>0.06</v>
+      </c>
+      <c r="D64">
+        <v>0.06</v>
+      </c>
+      <c r="E64">
+        <v>0.06</v>
+      </c>
+      <c r="F64">
+        <v>0.06</v>
+      </c>
+      <c r="G64">
+        <v>0.054000000000000006</v>
+      </c>
+      <c r="H64">
+        <v>0.054000000000000006</v>
+      </c>
+      <c r="I64" t="str">
+        <v/>
+      </c>
+      <c r="J64">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="str">
+        <v>Scourge III 9</v>
+      </c>
+      <c r="B65" t="str">
+        <v>Hunter Lethality</v>
+      </c>
+      <c r="C65">
+        <v>0.06</v>
+      </c>
+      <c r="D65">
+        <v>0.06</v>
+      </c>
+      <c r="E65">
+        <v>0.06</v>
+      </c>
+      <c r="F65">
+        <v>0.06</v>
+      </c>
+      <c r="G65">
+        <v>0.06</v>
+      </c>
+      <c r="H65">
+        <v>0.054000000000000006</v>
+      </c>
+      <c r="I65" t="str">
+        <v>Rally Capacity</v>
+      </c>
+      <c r="J65">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="str">
+        <v>Scourge III 10</v>
+      </c>
+      <c r="B66" t="str">
+        <v>Hunter Health</v>
+      </c>
+      <c r="C66">
+        <v>0.06</v>
+      </c>
+      <c r="D66">
+        <v>0.06</v>
+      </c>
+      <c r="E66">
+        <v>0.06</v>
+      </c>
+      <c r="F66">
+        <v>0.06</v>
+      </c>
+      <c r="G66">
+        <v>0.06</v>
+      </c>
+      <c r="H66">
+        <v>0.06</v>
+      </c>
+      <c r="I66" t="str">
+        <v>Adapt &amp; Overcome</v>
+      </c>
+      <c r="J66">
+        <v>40</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J66"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>